<commit_message>
feat: Add scoring script for Fixed-tab trials with visual feedback
</commit_message>
<xml_diff>
--- a/SmolVLA_eval_scoresheet.xlsx
+++ b/SmolVLA_eval_scoresheet.xlsx
@@ -427,7 +427,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F64"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -591,6 +591,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -601,6 +611,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -611,6 +631,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -621,6 +651,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -631,6 +671,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -641,6 +691,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -651,6 +711,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -661,6 +731,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -671,6 +751,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -681,6 +771,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -691,6 +791,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -701,6 +811,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -711,6 +831,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -721,6 +851,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -731,6 +871,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -741,6 +891,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -751,6 +911,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -761,6 +931,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -771,6 +951,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -781,6 +971,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -791,6 +991,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -801,6 +1011,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -811,6 +1031,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -821,6 +1051,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -831,6 +1071,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -841,6 +1091,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -851,6 +1111,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -861,6 +1131,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -871,6 +1151,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -881,6 +1171,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -891,6 +1191,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -901,6 +1211,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -911,6 +1231,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -921,6 +1251,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -931,6 +1271,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -941,6 +1291,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -951,6 +1311,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -961,6 +1331,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -971,6 +1351,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -981,6 +1371,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -991,6 +1391,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1001,6 +1411,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1011,6 +1431,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1021,6 +1451,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1031,6 +1471,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1041,6 +1491,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1051,6 +1511,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1061,6 +1531,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1071,6 +1551,16 @@
           <t>(0,0)</t>
         </is>
       </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1079,6 +1569,16 @@
       <c r="B64" t="inlineStr">
         <is>
           <t>(0,0)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1594,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G64"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>

</xml_diff>